<commit_message>
Update ETF pipeline outputs and scraper fixes
</commit_message>
<xml_diff>
--- a/providers/amundi/2026-07-06/amundi_etf_export.xlsx
+++ b/providers/amundi/2026-07-06/amundi_etf_export.xlsx
@@ -3470,7 +3470,7 @@
     <t>LU1708330235</t>
   </si>
   <si>
-    <t>4,009.5 M EUR</t>
+    <t>4,108.71 M EUR</t>
   </si>
   <si>
     <t>-0.60 %</t>
@@ -3551,7 +3551,7 @@
     <t>LU2355200796</t>
   </si>
   <si>
-    <t>3,430.73 M GBP</t>
+    <t>3,519.73 M GBP</t>
   </si>
   <si>
     <t>0.34 %</t>
@@ -3617,7 +3617,7 @@
     <t>LU2469335538</t>
   </si>
   <si>
-    <t>4,588.08 M USD</t>
+    <t>4,701.4 M USD</t>
   </si>
   <si>
     <t>0.31 %</t>
@@ -9199,7 +9199,7 @@
     <t>LU1806495575</t>
   </si>
   <si>
-    <t>1,101.64 M USD</t>
+    <t>1,102.02 M USD</t>
   </si>
   <si>
     <t>3.86 %</t>
@@ -9234,7 +9234,7 @@
     <t>LU2297533809</t>
   </si>
   <si>
-    <t>962.72 M EUR</t>
+    <t>963.09 M EUR</t>
   </si>
   <si>
     <t>-0.45 %</t>
@@ -10899,7 +10899,7 @@
     <t>0.17 %</t>
   </si>
   <si>
-    <t>859.97 M USD</t>
+    <t>859.79 M USD</t>
   </si>
   <si>
     <t>4.25 %</t>
@@ -11528,7 +11528,7 @@
     <t>LU1681041205</t>
   </si>
   <si>
-    <t>723.13 M USD</t>
+    <t>723.12 M USD</t>
   </si>
   <si>
     <t>2.21 %</t>
@@ -11569,7 +11569,7 @@
     <t>0.27 %</t>
   </si>
   <si>
-    <t>631.94 M EUR</t>
+    <t>631.96 M EUR</t>
   </si>
   <si>
     <t>1.21 %</t>
@@ -11632,7 +11632,7 @@
     <t>LU3307281595</t>
   </si>
   <si>
-    <t>540.72 M GBP</t>
+    <t>541.36 M GBP</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -18150,7 +18150,7 @@
     <t>LU2089239276</t>
   </si>
   <si>
-    <t>193.24 M USD</t>
+    <t>193.31 M USD</t>
   </si>
   <si>
     <t>3.96 %</t>
@@ -18214,7 +18214,7 @@
     <t>LU2621112452</t>
   </si>
   <si>
-    <t>144.49 M GBP</t>
+    <t>144.72 M GBP</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -18245,7 +18245,7 @@
     <t>LU2977997381</t>
   </si>
   <si>
-    <t>168.87 M EUR</t>
+    <t>168.94 M EUR</t>
   </si>
   <si>
     <t>-0.59 %</t>
@@ -18959,6 +18959,150 @@
 https://www.amundietf.co.uk/pdfDocuments/prospectus/FR0011720911/ENG/GBR/20260312</t>
   </si>
   <si>
+    <t>FEDG LN</t>
+  </si>
+  <si>
+    <t>Amundi USD Fed Funds Rate UCITS ETF Acc</t>
+  </si>
+  <si>
+    <t>LU1233598447</t>
+  </si>
+  <si>
+    <t>151.74 M USD</t>
+  </si>
+  <si>
+    <t>14.65 %</t>
+  </si>
+  <si>
+    <t>19.27 %</t>
+  </si>
+  <si>
+    <t>25.60 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/LU1233598447/ENG/GBR/INSTITUTIONNEL/ETF
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/LU1233598447/ENG/GBR/INSTITUTIONNEL/ETF/20260531
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/LU1233598447/ENG/GBR/INSTITUTIONNEL/ETF/20260430
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/LU1233598447/ENG/GBR/INSTITUTIONNEL/ETF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/kiid/LU1233598447/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/kiid/LU1233598447/ENG/GBR/20260211</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR/20260609
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR/20260511
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR/20260324</t>
+  </si>
+  <si>
+    <t>C101 GY</t>
+  </si>
+  <si>
+    <t>Amundi USD Fed Funds Rate UCITS ETF Dist</t>
+  </si>
+  <si>
+    <t>LU2090062352</t>
+  </si>
+  <si>
+    <t>3.87 %</t>
+  </si>
+  <si>
+    <t>19.28 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/kiid/LU2090062352/ENG/GBR/20260211
+https://www.amundietf.co.uk/pdfDocuments/kiid/LU2090062352/ENG/GBR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR/20260609
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR/20260511
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR/20260324</t>
+  </si>
+  <si>
+    <t>XMGA LN</t>
+  </si>
+  <si>
+    <t>Amundi MSCI USA Ex Mega Cap UCITS ETF Acc</t>
+  </si>
+  <si>
+    <t>IE000XL4IXU1</t>
+  </si>
+  <si>
+    <t>151.09 M USD</t>
+  </si>
+  <si>
+    <t>10.33 %</t>
+  </si>
+  <si>
+    <t>14.31 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF/20260531
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF/20260430
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF/20260331
+https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/kiid/IE000XL4IXU1/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/kiid/IE000XL4IXU1/ENG/GBR/20260218</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR/20260514
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR/20260407
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR/20260407
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR</t>
+  </si>
+  <si>
+    <t>MWON GY</t>
+  </si>
+  <si>
+    <t>Amundi S&amp;P SmallCap 600 Screened UCITS ETF DIST</t>
+  </si>
+  <si>
+    <t>IE000XLJ2JQ9</t>
+  </si>
+  <si>
+    <t>145.32 M USD</t>
+  </si>
+  <si>
+    <t>24.57 %</t>
+  </si>
+  <si>
+    <t>45.45 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/kiid/IE000XLJ2JQ9/ENG/GBR/20260218
+https://www.amundietf.co.uk/pdfDocuments/kiid/IE000XLJ2JQ9/ENG/GBR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR/20260514
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR/20260407
+https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR/20260407</t>
+  </si>
+  <si>
     <t>USIX LN</t>
   </si>
   <si>
@@ -18968,7 +19112,7 @@
     <t>LU1285959703</t>
   </si>
   <si>
-    <t>152.33 M USD</t>
+    <t>144.75 M USD</t>
   </si>
   <si>
     <t>15.76 %</t>
@@ -19003,7 +19147,7 @@
     <t>LU1285960032</t>
   </si>
   <si>
-    <t>133.12 M EUR</t>
+    <t>126.5 M EUR</t>
   </si>
   <si>
     <t>-0.42 %</t>
@@ -19066,150 +19210,6 @@
 https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1285959885/ENG/GBR</t>
   </si>
   <si>
-    <t>FEDG LN</t>
-  </si>
-  <si>
-    <t>Amundi USD Fed Funds Rate UCITS ETF Acc</t>
-  </si>
-  <si>
-    <t>LU1233598447</t>
-  </si>
-  <si>
-    <t>151.74 M USD</t>
-  </si>
-  <si>
-    <t>14.65 %</t>
-  </si>
-  <si>
-    <t>19.27 %</t>
-  </si>
-  <si>
-    <t>25.60 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/LU1233598447/ENG/GBR/INSTITUTIONNEL/ETF
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/LU1233598447/ENG/GBR/INSTITUTIONNEL/ETF/20260531
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/LU1233598447/ENG/GBR/INSTITUTIONNEL/ETF/20260430
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/LU1233598447/ENG/GBR/INSTITUTIONNEL/ETF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/kiid/LU1233598447/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/kiid/LU1233598447/ENG/GBR/20260211</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR/20260609
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR/20260511
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU1233598447/ENG/GBR/20260324</t>
-  </si>
-  <si>
-    <t>C101 GY</t>
-  </si>
-  <si>
-    <t>Amundi USD Fed Funds Rate UCITS ETF Dist</t>
-  </si>
-  <si>
-    <t>LU2090062352</t>
-  </si>
-  <si>
-    <t>3.87 %</t>
-  </si>
-  <si>
-    <t>19.28 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/kiid/LU2090062352/ENG/GBR/20260211
-https://www.amundietf.co.uk/pdfDocuments/kiid/LU2090062352/ENG/GBR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR/20260609
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR/20260511
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/LU2090062352/ENG/GBR/20260324</t>
-  </si>
-  <si>
-    <t>XMGA LN</t>
-  </si>
-  <si>
-    <t>Amundi MSCI USA Ex Mega Cap UCITS ETF Acc</t>
-  </si>
-  <si>
-    <t>IE000XL4IXU1</t>
-  </si>
-  <si>
-    <t>151.09 M USD</t>
-  </si>
-  <si>
-    <t>10.33 %</t>
-  </si>
-  <si>
-    <t>14.31 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF/20260531
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF/20260430
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF/20260331
-https://www.amundietf.co.uk/pdfDocuments/monthly-factsheet/IE000XL4IXU1/ENG/GBR/INSTITUTIONNEL/ETF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/kiid/IE000XL4IXU1/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/kiid/IE000XL4IXU1/ENG/GBR/20260218</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR/20260514
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR/20260407
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR/20260407
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XL4IXU1/ENG/GBR</t>
-  </si>
-  <si>
-    <t>MWON GY</t>
-  </si>
-  <si>
-    <t>Amundi S&amp;P SmallCap 600 Screened UCITS ETF DIST</t>
-  </si>
-  <si>
-    <t>IE000XLJ2JQ9</t>
-  </si>
-  <si>
-    <t>145.32 M USD</t>
-  </si>
-  <si>
-    <t>24.57 %</t>
-  </si>
-  <si>
-    <t>45.45 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/kiid/IE000XLJ2JQ9/ENG/GBR/20260218
-https://www.amundietf.co.uk/pdfDocuments/kiid/IE000XLJ2JQ9/ENG/GBR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR/20260514
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR/20260407
-https://www.amundietf.co.uk/pdfDocuments/prospectus/IE000XLJ2JQ9/ENG/GBR/20260407</t>
-  </si>
-  <si>
     <t>C051 GY</t>
   </si>
   <si>
@@ -21519,7 +21519,7 @@
     <t>LU2089239193</t>
   </si>
   <si>
-    <t>30.48 M USD</t>
+    <t>30.49 M USD</t>
   </si>
   <si>
     <t>0.26 %</t>
@@ -27987,7 +27987,7 @@
         <v>29</v>
       </c>
       <c r="I101" s="9">
-        <v>46.6238</v>
+        <v>46.6264</v>
       </c>
       <c r="J101" s="9" t="s">
         <v>862</v>
@@ -28040,7 +28040,7 @@
         <v>29</v>
       </c>
       <c r="I102" s="9">
-        <v>45.4364</v>
+        <v>45.4275</v>
       </c>
       <c r="J102" s="9" t="s">
         <v>872</v>
@@ -28093,7 +28093,7 @@
         <v>29</v>
       </c>
       <c r="I103" s="9">
-        <v>43.9289</v>
+        <v>43.933</v>
       </c>
       <c r="J103" s="9" t="s">
         <v>883</v>
@@ -28146,7 +28146,7 @@
         <v>29</v>
       </c>
       <c r="I104" s="9">
-        <v>43.237</v>
+        <v>43.2285</v>
       </c>
       <c r="J104" s="9" t="s">
         <v>872</v>
@@ -28199,7 +28199,7 @@
         <v>29</v>
       </c>
       <c r="I105" s="9">
-        <v>53.0425</v>
+        <v>53.0477</v>
       </c>
       <c r="J105" s="9" t="s">
         <v>899</v>
@@ -35884,7 +35884,7 @@
         <v>503</v>
       </c>
       <c r="I250" s="9">
-        <v>62.7441</v>
+        <v>62.7684</v>
       </c>
       <c r="J250" s="9" t="s">
         <v>1455</v>
@@ -35937,7 +35937,7 @@
         <v>503</v>
       </c>
       <c r="I251" s="9">
-        <v>38.8428</v>
+        <v>38.8562</v>
       </c>
       <c r="J251" s="9" t="s">
         <v>2290</v>
@@ -38110,7 +38110,7 @@
         <v>29</v>
       </c>
       <c r="I292" s="9">
-        <v>10.7135</v>
+        <v>10.714</v>
       </c>
       <c r="J292" s="9" t="s">
         <v>1980</v>
@@ -38163,7 +38163,7 @@
         <v>29</v>
       </c>
       <c r="I293" s="9">
-        <v>10.471</v>
+        <v>10.4714</v>
       </c>
       <c r="J293" s="9" t="s">
         <v>1980</v>
@@ -38905,7 +38905,7 @@
         <v>29</v>
       </c>
       <c r="I307" s="9">
-        <v>156.03</v>
+        <v>156.13</v>
       </c>
       <c r="J307" s="9" t="s">
         <v>2873</v>
@@ -38958,7 +38958,7 @@
         <v>29</v>
       </c>
       <c r="I308" s="9">
-        <v>65.92</v>
+        <v>65.97</v>
       </c>
       <c r="J308" s="9" t="s">
         <v>2884</v>
@@ -39011,7 +39011,7 @@
         <v>29</v>
       </c>
       <c r="I309" s="9">
-        <v>81.22</v>
+        <v>81.28</v>
       </c>
       <c r="J309" s="9" t="s">
         <v>2532</v>
@@ -48180,7 +48180,7 @@
         <v>29</v>
       </c>
       <c r="I482" s="9">
-        <v>21.7223</v>
+        <v>21.7312</v>
       </c>
       <c r="J482" s="9" t="s">
         <v>3702</v>
@@ -48233,7 +48233,7 @@
         <v>29</v>
       </c>
       <c r="I483" s="9">
-        <v>17.7409</v>
+        <v>17.7482</v>
       </c>
       <c r="J483" s="9" t="s">
         <v>3702</v>
@@ -48286,7 +48286,7 @@
         <v>29</v>
       </c>
       <c r="I484" s="9">
-        <v>10.6332</v>
+        <v>10.6375</v>
       </c>
       <c r="J484" s="9" t="s">
         <v>1120</v>
@@ -48339,7 +48339,7 @@
         <v>29</v>
       </c>
       <c r="I485" s="9">
-        <v>10.2772</v>
+        <v>10.2809</v>
       </c>
       <c r="J485" s="9" t="s">
         <v>4533</v>
@@ -49337,40 +49337,40 @@
         <v>26</v>
       </c>
       <c r="F504" s="9" t="s">
-        <v>188</v>
+        <v>143</v>
       </c>
       <c r="G504" s="9" t="s">
         <v>4715</v>
       </c>
       <c r="H504" s="9" t="s">
-        <v>503</v>
+        <v>29</v>
       </c>
       <c r="I504" s="9">
-        <v>94.643</v>
+        <v>125.9023</v>
       </c>
       <c r="J504" s="9" t="s">
-        <v>2176</v>
+        <v>4534</v>
       </c>
       <c r="K504" s="9" t="s">
-        <v>1804</v>
+        <v>2281</v>
       </c>
       <c r="L504" s="9" t="s">
         <v>4716</v>
       </c>
       <c r="M504" s="9" t="s">
-        <v>2750</v>
+        <v>4717</v>
       </c>
       <c r="N504" s="9" t="s">
-        <v>4717</v>
+        <v>4718</v>
       </c>
       <c r="O504" s="9" t="s">
-        <v>4718</v>
+        <v>4719</v>
       </c>
       <c r="P504" s="9" t="s">
-        <v>4719</v>
+        <v>4720</v>
       </c>
       <c r="Q504" s="9" t="s">
-        <v>4720</v>
+        <v>4721</v>
       </c>
     </row>
     <row r="505" spans="1:17" x14ac:dyDescent="0.25">
@@ -49378,52 +49378,52 @@
         <v>6</v>
       </c>
       <c r="B505" s="9" t="s">
-        <v>4721</v>
+        <v>4722</v>
       </c>
       <c r="C505" s="9" t="s">
-        <v>4722</v>
+        <v>4723</v>
       </c>
       <c r="D505" s="9" t="s">
-        <v>4723</v>
+        <v>4724</v>
       </c>
       <c r="E505" s="9" t="s">
-        <v>50</v>
+        <v>26</v>
       </c>
       <c r="F505" s="9" t="s">
-        <v>476</v>
+        <v>143</v>
       </c>
       <c r="G505" s="9" t="s">
-        <v>4724</v>
+        <v>4715</v>
       </c>
       <c r="H505" s="9" t="s">
-        <v>503</v>
+        <v>29</v>
       </c>
       <c r="I505" s="9">
-        <v>73.8454</v>
+        <v>104.9897</v>
       </c>
       <c r="J505" s="9" t="s">
+        <v>1925</v>
+      </c>
+      <c r="K505" s="9" t="s">
         <v>4725</v>
       </c>
-      <c r="K505" s="9" t="s">
+      <c r="L505" s="9" t="s">
+        <v>4716</v>
+      </c>
+      <c r="M505" s="9" t="s">
         <v>4726</v>
       </c>
-      <c r="L505" s="9" t="s">
+      <c r="N505" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="O505" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="P505" s="9" t="s">
         <v>4727</v>
       </c>
-      <c r="M505" s="9" t="s">
+      <c r="Q505" s="9" t="s">
         <v>4728</v>
-      </c>
-      <c r="N505" s="9" t="s">
-        <v>4729</v>
-      </c>
-      <c r="O505" s="9" t="s">
-        <v>4730</v>
-      </c>
-      <c r="P505" s="9" t="s">
-        <v>4731</v>
-      </c>
-      <c r="Q505" s="9" t="s">
-        <v>4732</v>
       </c>
     </row>
     <row r="506" spans="1:17" x14ac:dyDescent="0.25">
@@ -49431,52 +49431,52 @@
         <v>6</v>
       </c>
       <c r="B506" s="9" t="s">
-        <v>4733</v>
+        <v>4729</v>
       </c>
       <c r="C506" s="9" t="s">
-        <v>4734</v>
+        <v>4730</v>
       </c>
       <c r="D506" s="9" t="s">
-        <v>4735</v>
+        <v>4731</v>
       </c>
       <c r="E506" s="9" t="s">
         <v>26</v>
       </c>
       <c r="F506" s="9" t="s">
-        <v>188</v>
+        <v>132</v>
       </c>
       <c r="G506" s="9" t="s">
-        <v>4715</v>
+        <v>4732</v>
       </c>
       <c r="H506" s="9" t="s">
-        <v>503</v>
+        <v>29</v>
       </c>
       <c r="I506" s="9">
-        <v>10.1747</v>
+        <v>11.8576</v>
       </c>
       <c r="J506" s="9" t="s">
-        <v>2176</v>
+        <v>4733</v>
       </c>
       <c r="K506" s="9" t="s">
-        <v>1804</v>
+        <v>4734</v>
       </c>
       <c r="L506" s="9" t="s">
-        <v>4716</v>
+        <v>68</v>
       </c>
       <c r="M506" s="9" t="s">
-        <v>3111</v>
+        <v>68</v>
       </c>
       <c r="N506" s="9" t="s">
         <v>68</v>
       </c>
       <c r="O506" s="9" t="s">
+        <v>4735</v>
+      </c>
+      <c r="P506" s="9" t="s">
         <v>4736</v>
       </c>
-      <c r="P506" s="9" t="s">
+      <c r="Q506" s="9" t="s">
         <v>4737</v>
-      </c>
-      <c r="Q506" s="9" t="s">
-        <v>4738</v>
       </c>
     </row>
     <row r="507" spans="1:17" x14ac:dyDescent="0.25">
@@ -49484,52 +49484,52 @@
         <v>6</v>
       </c>
       <c r="B507" s="9" t="s">
+        <v>4738</v>
+      </c>
+      <c r="C507" s="9" t="s">
         <v>4739</v>
       </c>
-      <c r="C507" s="9" t="s">
+      <c r="D507" s="9" t="s">
         <v>4740</v>
-      </c>
-      <c r="D507" s="9" t="s">
-        <v>4741</v>
       </c>
       <c r="E507" s="9" t="s">
         <v>26</v>
       </c>
       <c r="F507" s="9" t="s">
-        <v>143</v>
+        <v>1120</v>
       </c>
       <c r="G507" s="9" t="s">
+        <v>4741</v>
+      </c>
+      <c r="H507" s="9" t="s">
+        <v>503</v>
+      </c>
+      <c r="I507" s="9">
+        <v>87.3557</v>
+      </c>
+      <c r="J507" s="9" t="s">
+        <v>4644</v>
+      </c>
+      <c r="K507" s="9" t="s">
         <v>4742</v>
-      </c>
-      <c r="H507" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="I507" s="9">
-        <v>125.9023</v>
-      </c>
-      <c r="J507" s="9" t="s">
-        <v>4534</v>
-      </c>
-      <c r="K507" s="9" t="s">
-        <v>2281</v>
       </c>
       <c r="L507" s="9" t="s">
         <v>4743</v>
       </c>
       <c r="M507" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="N507" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="O507" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="P507" s="9" t="s">
         <v>4744</v>
       </c>
-      <c r="N507" s="9" t="s">
+      <c r="Q507" s="9" t="s">
         <v>4745</v>
-      </c>
-      <c r="O507" s="9" t="s">
-        <v>4746</v>
-      </c>
-      <c r="P507" s="9" t="s">
-        <v>4747</v>
-      </c>
-      <c r="Q507" s="9" t="s">
-        <v>4748</v>
       </c>
     </row>
     <row r="508" spans="1:17" x14ac:dyDescent="0.25">
@@ -49537,52 +49537,52 @@
         <v>6</v>
       </c>
       <c r="B508" s="9" t="s">
-        <v>4749</v>
+        <v>4746</v>
       </c>
       <c r="C508" s="9" t="s">
-        <v>4750</v>
+        <v>4747</v>
       </c>
       <c r="D508" s="9" t="s">
-        <v>4751</v>
+        <v>4748</v>
       </c>
       <c r="E508" s="9" t="s">
         <v>26</v>
       </c>
       <c r="F508" s="9" t="s">
-        <v>143</v>
+        <v>188</v>
       </c>
       <c r="G508" s="9" t="s">
-        <v>4742</v>
+        <v>4749</v>
       </c>
       <c r="H508" s="9" t="s">
-        <v>29</v>
+        <v>503</v>
       </c>
       <c r="I508" s="9">
-        <v>104.9897</v>
+        <v>94.682</v>
       </c>
       <c r="J508" s="9" t="s">
-        <v>1925</v>
+        <v>2176</v>
       </c>
       <c r="K508" s="9" t="s">
+        <v>1804</v>
+      </c>
+      <c r="L508" s="9" t="s">
+        <v>4750</v>
+      </c>
+      <c r="M508" s="9" t="s">
+        <v>2750</v>
+      </c>
+      <c r="N508" s="9" t="s">
+        <v>4751</v>
+      </c>
+      <c r="O508" s="9" t="s">
         <v>4752</v>
       </c>
-      <c r="L508" s="9" t="s">
-        <v>4743</v>
-      </c>
-      <c r="M508" s="9" t="s">
+      <c r="P508" s="9" t="s">
         <v>4753</v>
       </c>
-      <c r="N508" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="O508" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="P508" s="9" t="s">
+      <c r="Q508" s="9" t="s">
         <v>4754</v>
-      </c>
-      <c r="Q508" s="9" t="s">
-        <v>4755</v>
       </c>
     </row>
     <row r="509" spans="1:17" x14ac:dyDescent="0.25">
@@ -49590,52 +49590,52 @@
         <v>6</v>
       </c>
       <c r="B509" s="9" t="s">
+        <v>4755</v>
+      </c>
+      <c r="C509" s="9" t="s">
         <v>4756</v>
       </c>
-      <c r="C509" s="9" t="s">
+      <c r="D509" s="9" t="s">
         <v>4757</v>
       </c>
-      <c r="D509" s="9" t="s">
+      <c r="E509" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F509" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="G509" s="9" t="s">
         <v>4758</v>
       </c>
-      <c r="E509" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="F509" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="G509" s="9" t="s">
+      <c r="H509" s="9" t="s">
+        <v>503</v>
+      </c>
+      <c r="I509" s="9">
+        <v>73.8724</v>
+      </c>
+      <c r="J509" s="9" t="s">
         <v>4759</v>
       </c>
-      <c r="H509" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="I509" s="9">
-        <v>11.8576</v>
-      </c>
-      <c r="J509" s="9" t="s">
+      <c r="K509" s="9" t="s">
         <v>4760</v>
       </c>
-      <c r="K509" s="9" t="s">
+      <c r="L509" s="9" t="s">
         <v>4761</v>
       </c>
-      <c r="L509" s="9" t="s">
-        <v>68</v>
-      </c>
       <c r="M509" s="9" t="s">
-        <v>68</v>
+        <v>4762</v>
       </c>
       <c r="N509" s="9" t="s">
-        <v>68</v>
+        <v>4763</v>
       </c>
       <c r="O509" s="9" t="s">
-        <v>4762</v>
+        <v>4764</v>
       </c>
       <c r="P509" s="9" t="s">
-        <v>4763</v>
+        <v>4765</v>
       </c>
       <c r="Q509" s="9" t="s">
-        <v>4764</v>
+        <v>4766</v>
       </c>
     </row>
     <row r="510" spans="1:17" x14ac:dyDescent="0.25">
@@ -49643,46 +49643,46 @@
         <v>6</v>
       </c>
       <c r="B510" s="9" t="s">
-        <v>4765</v>
+        <v>4767</v>
       </c>
       <c r="C510" s="9" t="s">
-        <v>4766</v>
+        <v>4768</v>
       </c>
       <c r="D510" s="9" t="s">
-        <v>4767</v>
+        <v>4769</v>
       </c>
       <c r="E510" s="9" t="s">
         <v>26</v>
       </c>
       <c r="F510" s="9" t="s">
-        <v>1120</v>
+        <v>188</v>
       </c>
       <c r="G510" s="9" t="s">
-        <v>4768</v>
+        <v>4749</v>
       </c>
       <c r="H510" s="9" t="s">
         <v>503</v>
       </c>
       <c r="I510" s="9">
-        <v>87.3557</v>
+        <v>10.1789</v>
       </c>
       <c r="J510" s="9" t="s">
-        <v>4644</v>
+        <v>2176</v>
       </c>
       <c r="K510" s="9" t="s">
-        <v>4769</v>
+        <v>1804</v>
       </c>
       <c r="L510" s="9" t="s">
+        <v>4750</v>
+      </c>
+      <c r="M510" s="9" t="s">
+        <v>3111</v>
+      </c>
+      <c r="N510" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="O510" s="9" t="s">
         <v>4770</v>
-      </c>
-      <c r="M510" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="N510" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="O510" s="9" t="s">
-        <v>68</v>
       </c>
       <c r="P510" s="9" t="s">
         <v>4771</v>
@@ -52950,7 +52950,7 @@
         <v>29</v>
       </c>
       <c r="I572" s="9">
-        <v>20.4213</v>
+        <v>20.4273</v>
       </c>
       <c r="J572" s="9" t="s">
         <v>5355</v>
@@ -53003,7 +53003,7 @@
         <v>29</v>
       </c>
       <c r="I573" s="9">
-        <v>18.8451</v>
+        <v>18.8506</v>
       </c>
       <c r="J573" s="9" t="s">
         <v>5355</v>
@@ -54805,7 +54805,7 @@
         <v>503</v>
       </c>
       <c r="I607" s="9">
-        <v>20.4728</v>
+        <v>20.4525</v>
       </c>
       <c r="J607" s="9" t="s">
         <v>4925</v>

</xml_diff>